<commit_message>
feat: 新增 LTCTask 及 LTCServiceRequest Profile，升級 TW Core 至 1.0.0
- 新增 LTCTask Profile（繼承 FHIR R4 Task）支援轉介確認與計畫狀態更新
- 新增 LTCServiceRequest Profile（繼承 TW Core ServiceRequest）支援轉介申請與服務請求
- 升級依賴 tw.gov.mohw.twcore 從 0.3.2 至 1.0.0
- 更新網頁文件（profiles-and-extensions、examples、index）
- 新增範例：轉介確認任務、長照轉介服務請求
- 更新 ignoreWarnings.txt 抑制繼承的 v2-0116 版本警告
- 更新 IG 網頁（0 errors, 0 warnings）
</commit_message>
<xml_diff>
--- a/docs/StructureDefinition-LTC-CarePlan-CS100.xlsx
+++ b/docs/StructureDefinition-LTC-CarePlan-CS100.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2677" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2680" uniqueCount="531">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-02T02:26:08+08:00</t>
+    <t>2026-04-02T13:32:15+08:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -263,10 +263,10 @@
 </t>
   </si>
   <si>
-    <t>Healthcare plan for patient or group</t>
-  </si>
-  <si>
-    <t>Describes the intention of how one or more practitioners intend to deliver care for a particular patient, group or community for a period of time, possibly limited to care for a specific condition or set of conditions.</t>
+    <t>特定照護目標下為一位患者或一群患者識別的活動、干預和結果計畫</t>
+  </si>
+  <si>
+    <t>描述為實現一個或多個目標而將為一位患者(或一群患者)進行的活動的計畫，包括診斷、監測、評估、治療、藥物治療、追蹤等。</t>
   </si>
   <si>
     <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
@@ -292,13 +292,13 @@
 </t>
   </si>
   <si>
-    <t>Logical id of this artifact</t>
-  </si>
-  <si>
-    <t>The logical id of the resource, as used in the URL for the resource. Once assigned, this value never changes.</t>
-  </si>
-  <si>
-    <t>The only time that a resource does not have an id is when it is being submitted to the server using a create operation.</t>
+    <t>不重複的 ID 用以識別儲存在特定 FHIR Server 中的 CarePlan 紀錄，通常又稱為邏輯性 ID。</t>
+  </si>
+  <si>
+    <t>resource 的邏輯 ID，在 resource 的 URL 中使用。一旦指定，這個值永遠不會改變。</t>
+  </si>
+  <si>
+    <t>一個 resource 使用新增操作(create operation)提交給伺服器時，此 resource 沒有 id，它的 id 在 resource 被創建後由伺器分配/指定。</t>
   </si>
   <si>
     <t>Resource.id</t>
@@ -311,10 +311,10 @@
 </t>
   </si>
   <si>
-    <t>Metadata about the resource</t>
-  </si>
-  <si>
-    <t>The metadata about the resource. This is content that is maintained by the infrastructure. Changes to the content might not always be associated with version changes to the resource.</t>
+    <t>此 CarePlan Resource 的 metadata</t>
+  </si>
+  <si>
+    <t>關於 resource 的 metadata。這是由基礎建設維護的內容。內容的更改可能並不總是與 resource 的版本更改相關聯。</t>
   </si>
   <si>
     <t>Resource.meta</t>
@@ -331,13 +331,13 @@
 </t>
   </si>
   <si>
-    <t>A set of rules under which this content was created</t>
-  </si>
-  <si>
-    <t>A reference to a set of rules that were followed when the resource was constructed, and which must be understood when processing the content. Often, this is a reference to an implementation guide that defines the special rules along with other profiles etc.</t>
-  </si>
-  <si>
-    <t>Asserting this rule set restricts the content to be only understood by a limited set of trading partners. This inherently limits the usefulness of the data in the long term. However, the existing health eco-system is highly fractured, and not yet ready to define, collect, and exchange data in a generally computable sense. Wherever possible, implementers and/or specification writers should avoid using this element. Often, when used, the URL is a reference to an implementation guide that defines these special rules as part of it's narrative along with other profiles, value sets, etc.</t>
+    <t>創建此內容所依據的一組規則</t>
+  </si>
+  <si>
+    <t>構建 resource 時遵循的一系列規則的參照，在處理內容時必須理解這些規則。通常這是對 IG 所定義之特殊規則及其他 profiles 的參照。</t>
+  </si>
+  <si>
+    <t>宣告這套規則限制了內容只能被有限的交易夥伴所理解。這從本質上限制了資料的長期有用性。然而，現有的健康生態體系高度分裂，還沒有準備好以普遍可計算的方式定義、收集和交換資料。只要有可能，實作者和/或規範編寫者應該避免使用這個資料項目。通常在使用時，此 URL 是對 IG 的參照，此 IG 將這些特殊規則與其他 profiles、value sets 等一起定義為其敘述的一部分。</t>
   </si>
   <si>
     <t>Resource.implicitRules</t>
@@ -350,19 +350,22 @@
 </t>
   </si>
   <si>
-    <t>Language of the resource content</t>
-  </si>
-  <si>
-    <t>The base language in which the resource is written.</t>
-  </si>
-  <si>
-    <t>Language is provided to support indexing and accessibility (typically, services such as text to speech use the language tag). The html language tag in the narrative applies  to the narrative. The language tag on the resource may be used to specify the language of other presentations generated from the data in the resource. Not all the content has to be in the base language. The Resource.language should not be assumed to apply to the narrative automatically. If a language is specified, it should it also be specified on the div element in the html (see rules in HTML5 for information about the relationship between xml:lang and the html lang attribute).</t>
+    <t>用以表述 CarePlan Resource 內容的語言</t>
+  </si>
+  <si>
+    <t>編寫此 resource 的語言</t>
+  </si>
+  <si>
+    <t>提供語言是為了支援索引和可存取性(通常，文字表述轉語音等服務使用此語言標籤)。html lanuage tag 適用於此敘述。resource 上的語言標籤可用於指定從 resource 中的資料所產成的其他表述之語言。不是所有的內容都必須使用此語言。不應該假定 Resource.language 自動適用於敘述。如果指定語言，它也應該被指定在 html 中的 div 資料項目(關於 xml:lang 和 html lang 屬性之間的關係，見 HTML5 中的規則)。</t>
+  </si>
+  <si>
+    <t>zh-TW</t>
   </si>
   <si>
     <t>preferred</t>
   </si>
   <si>
-    <t>A human language.</t>
+    <t>人類語言；鼓勵使用 CommonLanguages 代碼表中的代碼，但不強制一定要使用此代碼表，你也可使用其他代碼表的代碼或單純以文字表示。</t>
   </si>
   <si>
     <t>http://hl7.org/fhir/ValueSet/languages</t>
@@ -382,13 +385,13 @@
 </t>
   </si>
   <si>
-    <t>CarePlan Resource之內容摘要以供人閱讀</t>
-  </si>
-  <si>
-    <t>A human-readable narrative that contains a summary of the resource and can be used to represent the content of the resource to a human. The narrative need not encode all the structured data, but is required to contain sufficient detail to make it "clinically safe" for a human to just read the narrative. Resource definitions may define what content should be represented in the narrative to ensure clinical safety.</t>
-  </si>
-  <si>
-    <t>Contained resources do not have narrative. Resources that are not contained SHOULD have a narrative. In some cases, a resource may only have text with little or no additional discrete data (as long as all minOccurs=1 elements are satisfied).  This may be necessary for data from legacy systems where information is captured as a "text blob" or where text is additionally entered raw or narrated and encoded information is added later.</t>
+    <t>CarePlan Resource 之內容摘要以供人閱讀</t>
+  </si>
+  <si>
+    <t>人可讀的敘述，包含 resource 的摘要，可用於向人表述 resource 的內容。敘述不需要對所有的結構化資料進行編碼，但需要包含足夠的細節使人在閱讀敘述時理解「臨床安全性」。resource 定義有哪些內容應該在敘述中表示，以確保臨床安全。</t>
+  </si>
+  <si>
+    <t>內嵌(contained)的 resource 沒有敘述，非內嵌(contained)的 resource 則 **建議應該(SHOULD)** 有敘述。有時 resource 可能只有文字表述，很少或沒有額外的結構化資料(只要滿足所有 minOccurs=1 的資料項目)。這可能出現在舊系統的資料，當資訊以 「文字表述區塊(text blob)」的形式被取得，或者文字表述是原始輸入或說明，而編碼資訊稍後再添加。</t>
   </si>
   <si>
     <t>DomainResource.text</t>
@@ -465,7 +468,7 @@
     <t>required</t>
   </si>
   <si>
-    <t>Constrained value set of narrative statuses.</t>
+    <t>敘述狀態的受限值集。</t>
   </si>
   <si>
     <t>https://twcore.mohw.gov.tw/ig/twcore/ValueSet/narrative-status</t>
@@ -484,7 +487,7 @@
 </t>
   </si>
   <si>
-    <t>Limited xhtml content</t>
+    <t>有限的 xhtml 內容</t>
   </si>
   <si>
     <t>The actual narrative content, a stripped down version of XHTML.</t>
@@ -582,7 +585,7 @@
     <t>CarePlan.instantiatesCanonical</t>
   </si>
   <si>
-    <t xml:space="preserve">canonical(PlanDefinition|Questionnaire|Measure|ActivityDefinition|OperationDefinition)
+    <t xml:space="preserve">canonical(PlanDefinition|4.0.1|Questionnaire|4.0.1|Measure|4.0.1|ActivityDefinition|4.0.1|OperationDefinition|4.0.1)
 </t>
   </si>
   <si>
@@ -624,10 +627,13 @@
 </t>
   </si>
   <si>
-    <t>Fulfills CarePlan</t>
-  </si>
-  <si>
-    <t>A care plan that is fulfilled in whole or in part by this care plan.</t>
+    <t>履行或延伸的照護計畫</t>
+  </si>
+  <si>
+    <t>識別此照護計畫所建立的父計畫。</t>
+  </si>
+  <si>
+    <t>參照可以是相對的、絕對的或內部的。</t>
   </si>
   <si>
     <t>Allows tracing of the care plan and tracking whether proposals/recommendations were acted upon.</t>
@@ -643,13 +649,10 @@
 </t>
   </si>
   <si>
-    <t>CarePlan replaced by this CarePlan</t>
-  </si>
-  <si>
-    <t>Completed or terminated care plan whose function is taken by this new care plan.</t>
-  </si>
-  <si>
-    <t>The replacement could be because the initial care plan was immediately rejected (due to an issue) or because the previous care plan was completed, but the need for the action described by the care plan remains ongoing.</t>
+    <t>被此計畫取代的照護計畫</t>
+  </si>
+  <si>
+    <t>識別被此照護計畫所取代的照護計畫。</t>
   </si>
   <si>
     <t>Allows tracing the continuation of a therapy or administrative process instantiated through multiple care plans.</t>
@@ -661,26 +664,25 @@
     <t>CarePlan.partOf</t>
   </si>
   <si>
-    <t>Part of referenced CarePlan</t>
-  </si>
-  <si>
-    <t>A larger care plan of which this particular care plan is a component or step.</t>
-  </si>
-  <si>
-    <t>Each care plan is an independent request, such that having a care plan be part of another care plan can cause issues with cascading statuses.  As such, this element is still being discussed.</t>
+    <t>作為父照護計畫的一部分</t>
+  </si>
+  <si>
+    <t>此照護計畫是另一個照護計畫的一部分。例如，專門針對骨折修復或糖尿病控制的計畫可能是出院護理計畫的一部分。</t>
   </si>
   <si>
     <t>CarePlan.status</t>
   </si>
   <si>
-    <t>draft | active | on-hold | revoked | completed | entered-in-error | unknown</t>
-  </si>
-  <si>
-    <t>Indicates whether the plan is currently being acted upon, represents future intentions or is now a historical record.</t>
-  </si>
-  <si>
-    <t>The unknown code is not to be used to convey other statuses.  The unknown code should be used when one of the statuses applies, but the authoring system doesn't know the current state of the care plan.
-This element is labeled as a modifier because the status contains the code entered-in-error that marks the plan as not currently valid.</t>
+    <t>照護計畫目前的狀態</t>
+  </si>
+  <si>
+    <t>指明照護計畫是否正在執行中、表示未來意向或現在已成為歷史記錄。</t>
+  </si>
+  <si>
+    <t>可以在 [[event.html#statemachine | 事件模式]] 文件中找到一個標準的狀態轉換圖。「未知」不代表「其他」狀態 - 必須使用其中一個已定義的狀態，「未知」用於表示不確定當前狀態。</t>
+  </si>
+  <si>
+    <t>指出計畫是否正在實施、代表未來意圖或是現在的歷史記錄。</t>
   </si>
   <si>
     <t>http://hl7.org/fhir/ValueSet/request-status</t>
@@ -701,10 +703,10 @@
     <t>CarePlan.intent</t>
   </si>
   <si>
-    <t>proposal | plan | order | option</t>
-  </si>
-  <si>
-    <t>Indicates the level of authority/intentionality associated with the care plan and where the care plan fits into the workflow chain.</t>
+    <t>照護計畫的意圖</t>
+  </si>
+  <si>
+    <t>表示與照護計畫相關的權威性/意向性程度。</t>
   </si>
   <si>
     <t>This element is labeled as a modifier because the intent alters when and how the resource is actually applicable.</t>
@@ -716,7 +718,7 @@
     <t>plan</t>
   </si>
   <si>
-    <t>Codes indicating the degree of authority/intentionality associated with a care plan</t>
+    <t>表示與照護計畫相關的權威性/意向性程度的代碼</t>
   </si>
   <si>
     <t>http://hl7.org/fhir/ValueSet/care-plan-intent</t>
@@ -732,16 +734,16 @@
 </t>
   </si>
   <si>
-    <t>Type of plan</t>
-  </si>
-  <si>
-    <t>Type of plan.</t>
+    <t>照護計畫的類型</t>
+  </si>
+  <si>
+    <t>照護計畫的類型。</t>
   </si>
   <si>
     <t>There may be multiple axes of categorization and one plan may serve multiple purposes.  In some cases, this may be redundant with references to CarePlan.concern.</t>
   </si>
   <si>
-    <t>Identifies what "kind" of plan this is to support differentiation between multiple co-existing plans; e.g., "Home health", "psychiatric", "asthma", "disease management", "wellness plan", etc.</t>
+    <t>識別這是什麼「種類」的計畫，以支援多個共存計畫之間的區分；例如：「居家健康」、「精神科」、「氣喘」、「疾病管理」、「保健計畫」等。</t>
   </si>
   <si>
     <t>example</t>
@@ -750,7 +752,7 @@
     <t>Identifies what "kind" of plan this is to support differentiation between multiple co-existing plans; e.g. "Home health", "psychiatric", "asthma", "disease management", etc.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/care-plan-category</t>
+    <t>http://hl7.org/fhir/ValueSet/care-plan-category|4.0.1</t>
   </si>
   <si>
     <t xml:space="preserve">pattern:$this}
@@ -764,6 +766,9 @@
   </si>
   <si>
     <t>AssessPlan</t>
+  </si>
+  <si>
+    <t>評估計畫</t>
   </si>
   <si>
     <t>Identifies what "kind" of plan this is to support differentiation between multiple co-existing plans; e.g. "Home health", "psychiatric", "asthma", "disease management", "wellness plan", etc.</t>
@@ -815,13 +820,13 @@
 </t>
   </si>
   <si>
-    <t>Who the care plan is for</t>
-  </si>
-  <si>
-    <t>Who care plan is for.</t>
-  </si>
-  <si>
-    <t>Identifies the patient or group whose intended care is described by the plan.</t>
+    <t>照護計畫的對象</t>
+  </si>
+  <si>
+    <t>照護計畫是為了誰。</t>
+  </si>
+  <si>
+    <t>識別計畫描述其意圖照護的病人或群體。</t>
   </si>
   <si>
     <t>Request.subject</t>
@@ -843,13 +848,13 @@
 </t>
   </si>
   <si>
-    <t>Encounter created as part of</t>
-  </si>
-  <si>
-    <t>The Encounter during which this CarePlan was created or to which the creation of this record is tightly associated.</t>
-  </si>
-  <si>
-    <t>This will typically be the encounter the event occurred within, but some activities may be initiated prior to or after the official completion of an encounter but still be tied to the context of the encounter. CarePlan activities conducted as a result of the care plan may well occur as part of other encounters.</t>
+    <t>與此照護計畫相關的就醫事件</t>
+  </si>
+  <si>
+    <t>此照護計畫是在哪個就醫情境產生的。</t>
+  </si>
+  <si>
+    <t>參照可以是相對的、絕對的或內部的。注意：如果 Encounter 參照是一個 Episode of Care 的一部分，則此資料點不足以隱含建立關聯。</t>
   </si>
   <si>
     <t>Request.context</t>
@@ -987,13 +992,10 @@
 </t>
   </si>
   <si>
-    <t>Who is the designated responsible party</t>
-  </si>
-  <si>
-    <t>When populated, the author is responsible for the care plan.  The care plan is attributed to the author.</t>
-  </si>
-  <si>
-    <t>The author may also be a contributor.  For example, an organization can be an author, but not listed as a contributor.</t>
+    <t>照護計畫的作者</t>
+  </si>
+  <si>
+    <t>負責建立照護計畫內容的個人或組織。</t>
   </si>
   <si>
     <t>Request.requester</t>
@@ -1005,13 +1007,10 @@
     <t>CarePlan.contributor</t>
   </si>
   <si>
-    <t>Who provided the content of the care plan</t>
-  </si>
-  <si>
-    <t>Identifies the individual(s) or organization who provided the contents of the care plan.</t>
-  </si>
-  <si>
-    <t>Collaborative care plans may have multiple contributors.</t>
+    <t>對計畫提供資訊的人員</t>
+  </si>
+  <si>
+    <t>對照護計畫的建立提供資訊的個人或組織，但不對照護計畫負責。</t>
   </si>
   <si>
     <t>CarePlan.careTeam</t>
@@ -1021,10 +1020,10 @@
 </t>
   </si>
   <si>
-    <t>Who's involved in plan?</t>
-  </si>
-  <si>
-    <t>Identifies all people and organizations who are expected to be involved in the care envisioned by this plan.</t>
+    <t>執行照護工作的團隊</t>
+  </si>
+  <si>
+    <t>確定負責執行此照護計畫的照護團隊。</t>
   </si>
   <si>
     <t>Allows representation of care teams, helps scope care plan.  In some cases may be a determiner of access permissions.</t>
@@ -1043,13 +1042,10 @@
 </t>
   </si>
   <si>
-    <t>Health issues this plan addresses</t>
-  </si>
-  <si>
-    <t>Identifies the conditions/problems/concerns/diagnoses/etc. whose management and/or mitigation are handled by this plan.</t>
-  </si>
-  <si>
-    <t>When the diagnosis is related to an allergy or intolerance, the Condition and AllergyIntolerance resources can both be used. However, to be actionable for decision support, using Condition alone is not sufficient as the allergy or intolerance condition needs to be represented as an AllergyIntolerance.</t>
+    <t>本計畫處理的健康問題</t>
+  </si>
+  <si>
+    <t>本照護計畫試圖解決的健康問題(例如：疾病、病情、問題)。</t>
   </si>
   <si>
     <t>Links plan to the conditions it manages.  The element can identify risks addressed by the plan as well as active conditions.  (The Condition resource can include things like "at risk for hypertension" or "fall risk".)  Also scopes plans - multiple plans may exist addressing different concerns.</t>
@@ -1092,7 +1088,7 @@
     <t>CarePlan.goal</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Goal)
+    <t xml:space="preserve">Reference(Goal|4.0.1)
 </t>
   </si>
   <si>
@@ -1179,13 +1175,13 @@
     <t>Identifies the results of the activity.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/care-plan-activity-outcome</t>
+    <t>http://hl7.org/fhir/ValueSet/care-plan-activity-outcome|4.0.1</t>
   </si>
   <si>
     <t>CarePlan.activity.outcomeReference</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Resource)
+    <t xml:space="preserve">Reference(Resource|4.0.1)
 </t>
   </si>
   <si>
@@ -1239,14 +1235,10 @@
 </t>
   </si>
   <si>
-    <t>Activity details defined in specific resource</t>
-  </si>
-  <si>
-    <t>The details of the proposed activity represented in a specific resource.</t>
-  </si>
-  <si>
-    <t>Standard extension exists ([resource-pertainsToGoal](http://hl7.org/fhir/R4/extension-resource-pertainstogoal.html)) that allows goals to be referenced from any of the referenced resources in CarePlan.activity.reference.  -The goal should be visible when the resource referenced by CarePlan.activity.reference is viewed independently from the CarePlan.  Requests that are pointed to by a CarePlan using this element should *not* point to this CarePlan using the "basedOn" element.  i.e. Requests that are part of a CarePlan are not "based on" the CarePlan.</t>
+    <t>照護行動的明細</t>
+  </si>
+  <si>
+    <t>包含照護計畫之照護行動(診斷、治療等)明細的 request/request-like 資源。</t>
   </si>
   <si>
     <t>Details in a form consistent with other applications and contexts of use.</t>
@@ -1333,7 +1325,7 @@
     <t>CarePlan.activity.detail.instantiatesCanonical</t>
   </si>
   <si>
-    <t xml:space="preserve">canonical(PlanDefinition|ActivityDefinition|Questionnaire|Measure|OperationDefinition)
+    <t xml:space="preserve">canonical(PlanDefinition|4.0.1|ActivityDefinition|4.0.1|Questionnaire|4.0.1|Measure|4.0.1|OperationDefinition|4.0.1)
 </t>
   </si>
   <si>
@@ -1367,7 +1359,7 @@
     <t>Detailed description of the type of activity; e.g. What lab test, what procedure, what kind of encounter.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/procedure-code</t>
+    <t>http://hl7.org/fhir/ValueSet/procedure-code|4.0.1</t>
   </si>
   <si>
     <t>Request.code</t>
@@ -1394,7 +1386,7 @@
     <t>Identifies why a care plan activity is needed.  Can include any health condition codes as well as such concepts as "general wellness", prophylaxis, surgical preparation, etc.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/clinical-findings</t>
+    <t>http://hl7.org/fhir/ValueSet/clinical-findings|4.0.1</t>
   </si>
   <si>
     <t>Request.reasonCode</t>
@@ -1407,10 +1399,10 @@
 </t>
   </si>
   <si>
-    <t>Why activity is needed</t>
-  </si>
-  <si>
-    <t>Indicates another resource, such as the health condition(s), whose existence justifies this request and drove the inclusion of this particular activity as part of the plan.</t>
+    <t>為何需要此行動</t>
+  </si>
+  <si>
+    <t>指出為何此行動是此照護計畫的一部分。</t>
   </si>
   <si>
     <t>Conditions can be identified at the activity level that are not identified as reasons for the overall plan.</t>
@@ -1541,13 +1533,10 @@
 </t>
   </si>
   <si>
-    <t>Where it should happen</t>
-  </si>
-  <si>
-    <t>Identifies the facility where the activity will occur; e.g. home, hospital, specific clinic, etc.</t>
-  </si>
-  <si>
-    <t>May reference a specific clinical location or may identify a type of location.</t>
+    <t>行動發生的地點</t>
+  </si>
+  <si>
+    <t>預期要執行此行動的地點。</t>
   </si>
   <si>
     <t>Helps in planning of activity.</t>
@@ -1566,13 +1555,10 @@
 </t>
   </si>
   <si>
-    <t>Who will be responsible?</t>
-  </si>
-  <si>
-    <t>Identifies who's expected to be involved in the activity.</t>
-  </si>
-  <si>
-    <t>A performer MAY also be a participant in the care plan.</t>
+    <t>執行或提供此行動的人員</t>
+  </si>
+  <si>
+    <t>確定預期要執行此行動的特定人員或組織。</t>
   </si>
   <si>
     <t>Request.performer</t>
@@ -1588,7 +1574,7 @@
   </si>
   <si>
     <t>CodeableConcept
-Reference(Medication|Substance)</t>
+Reference(Medication|4.0.1|Substance|4.0.1)</t>
   </si>
   <si>
     <t>What is to be administered/supplied</t>
@@ -1600,7 +1586,7 @@
     <t>A product supplied or administered as part of a care plan activity.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/medication-codes</t>
+    <t>http://hl7.org/fhir/ValueSet/medication-codes|4.0.1</t>
   </si>
   <si>
     <t>.participation[typeCode=PRD].role</t>
@@ -1619,6 +1605,12 @@
 </t>
   </si>
   <si>
+    <t>物料/主題/產品資訊要參照的資源</t>
+  </si>
+  <si>
+    <t>辨識行動所涉及的物料/主題/產品。</t>
+  </si>
+  <si>
     <t>CarePlan.activity.detail.dailyAmount</t>
   </si>
   <si>
@@ -1626,7 +1618,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Quantity {SimpleQuantity}
+    <t xml:space="preserve">Quantity {SimpleQuantity|4.0.1}
 </t>
   </si>
   <si>
@@ -2670,7 +2662,7 @@
         <v>20</v>
       </c>
       <c r="T6" t="s" s="2">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="U6" t="s" s="2">
         <v>20</v>
@@ -2682,13 +2674,13 @@
         <v>20</v>
       </c>
       <c r="X6" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Y6" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="Z6" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="AA6" t="s" s="2">
         <v>20</v>
@@ -2706,7 +2698,7 @@
         <v>20</v>
       </c>
       <c r="AF6" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AG6" t="s" s="2">
         <v>78</v>
@@ -2735,14 +2727,14 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" t="s" s="2">
@@ -2761,16 +2753,16 @@
         <v>20</v>
       </c>
       <c r="K7" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="L7" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="N7" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="O7" s="2"/>
       <c r="P7" t="s" s="2">
@@ -2820,7 +2812,7 @@
         <v>20</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>78</v>
@@ -2838,7 +2830,7 @@
         <v>20</v>
       </c>
       <c r="AL7" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AM7" t="s" s="2">
         <v>20</v>
@@ -2849,10 +2841,10 @@
     </row>
     <row r="8" hidden="true">
       <c r="A8" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -2875,13 +2867,13 @@
         <v>20</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
@@ -2932,7 +2924,7 @@
         <v>20</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>78</v>
@@ -2950,7 +2942,7 @@
         <v>20</v>
       </c>
       <c r="AL8" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AM8" t="s" s="2">
         <v>20</v>
@@ -2961,14 +2953,14 @@
     </row>
     <row r="9" hidden="true">
       <c r="A9" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" t="s" s="2">
@@ -2987,16 +2979,16 @@
         <v>20</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="N9" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O9" s="2"/>
       <c r="P9" t="s" s="2">
@@ -3034,19 +3026,19 @@
         <v>20</v>
       </c>
       <c r="AB9" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AC9" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AD9" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE9" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>78</v>
@@ -3058,13 +3050,13 @@
         <v>20</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AK9" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL9" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AM9" t="s" s="2">
         <v>20</v>
@@ -3075,10 +3067,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
@@ -3104,10 +3096,10 @@
         <v>107</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -3134,13 +3126,13 @@
         <v>20</v>
       </c>
       <c r="X10" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Y10" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Z10" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="AA10" t="s" s="2">
         <v>20</v>
@@ -3158,7 +3150,7 @@
         <v>20</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>87</v>
@@ -3176,7 +3168,7 @@
         <v>20</v>
       </c>
       <c r="AL10" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AM10" t="s" s="2">
         <v>20</v>
@@ -3187,10 +3179,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -3213,16 +3205,16 @@
         <v>20</v>
       </c>
       <c r="K11" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="N11" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="O11" s="2"/>
       <c r="P11" t="s" s="2">
@@ -3272,7 +3264,7 @@
         <v>20</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>87</v>
@@ -3284,13 +3276,13 @@
         <v>20</v>
       </c>
       <c r="AJ11" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="AK11" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL11" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AM11" t="s" s="2">
         <v>20</v>
@@ -3301,14 +3293,14 @@
     </row>
     <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" t="s" s="2">
@@ -3327,16 +3319,16 @@
         <v>20</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N12" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="O12" s="2"/>
       <c r="P12" t="s" s="2">
@@ -3386,7 +3378,7 @@
         <v>20</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>78</v>
@@ -3404,7 +3396,7 @@
         <v>20</v>
       </c>
       <c r="AL12" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AM12" t="s" s="2">
         <v>20</v>
@@ -3415,14 +3407,14 @@
     </row>
     <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" t="s" s="2">
@@ -3441,16 +3433,16 @@
         <v>20</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -3500,7 +3492,7 @@
         <v>20</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>78</v>
@@ -3512,13 +3504,13 @@
         <v>20</v>
       </c>
       <c r="AJ13" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AK13" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AM13" t="s" s="2">
         <v>20</v>
@@ -3529,14 +3521,14 @@
     </row>
     <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" t="s" s="2">
@@ -3555,19 +3547,19 @@
         <v>20</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="N14" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O14" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="P14" t="s" s="2">
         <v>20</v>
@@ -3616,7 +3608,7 @@
         <v>20</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>78</v>
@@ -3628,13 +3620,13 @@
         <v>20</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AK14" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL14" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AM14" t="s" s="2">
         <v>20</v>
@@ -3645,10 +3637,10 @@
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -3671,19 +3663,19 @@
         <v>88</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="N15" t="s" s="2">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="O15" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P15" t="s" s="2">
         <v>20</v>
@@ -3732,7 +3724,7 @@
         <v>20</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>78</v>
@@ -3747,24 +3739,24 @@
         <v>99</v>
       </c>
       <c r="AK15" t="s" s="2">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AL15" t="s" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="AM15" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="AN15" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -3787,13 +3779,13 @@
         <v>88</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -3844,7 +3836,7 @@
         <v>20</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>78</v>
@@ -3859,10 +3851,10 @@
         <v>99</v>
       </c>
       <c r="AK16" t="s" s="2">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="AL16" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AM16" t="s" s="2">
         <v>20</v>
@@ -3873,10 +3865,10 @@
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3902,13 +3894,13 @@
         <v>101</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="N17" t="s" s="2">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
@@ -3958,7 +3950,7 @@
         <v>20</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>78</v>
@@ -3973,10 +3965,10 @@
         <v>99</v>
       </c>
       <c r="AK17" t="s" s="2">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="AL17" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AM17" t="s" s="2">
         <v>20</v>
@@ -3987,14 +3979,14 @@
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
@@ -4013,17 +4005,19 @@
         <v>88</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>195</v>
-      </c>
-      <c r="N18" s="2"/>
+        <v>196</v>
+      </c>
+      <c r="N18" t="s" s="2">
+        <v>197</v>
+      </c>
       <c r="O18" t="s" s="2">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="P18" t="s" s="2">
         <v>20</v>
@@ -4072,7 +4066,7 @@
         <v>20</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>78</v>
@@ -4087,7 +4081,7 @@
         <v>99</v>
       </c>
       <c r="AK18" t="s" s="2">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="AL18" t="s" s="2">
         <v>20</v>
@@ -4101,14 +4095,14 @@
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
@@ -4127,19 +4121,19 @@
         <v>88</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="O19" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="P19" t="s" s="2">
         <v>20</v>
@@ -4188,7 +4182,7 @@
         <v>20</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>78</v>
@@ -4203,7 +4197,7 @@
         <v>99</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AL19" t="s" s="2">
         <v>20</v>
@@ -4217,10 +4211,10 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -4243,16 +4237,16 @@
         <v>88</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="N20" t="s" s="2">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
@@ -4302,7 +4296,7 @@
         <v>20</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>78</v>
@@ -4369,7 +4363,7 @@
         <v>212</v>
       </c>
       <c r="O21" t="s" s="2">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="P21" t="s" s="2">
         <v>20</v>
@@ -4394,13 +4388,13 @@
         <v>20</v>
       </c>
       <c r="X21" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Y21" t="s" s="2">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="Z21" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AA21" t="s" s="2">
         <v>20</v>
@@ -4433,24 +4427,24 @@
         <v>99</v>
       </c>
       <c r="AK21" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AM21" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AN21" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -4476,16 +4470,16 @@
         <v>107</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="N22" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="O22" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="P22" t="s" s="2">
         <v>20</v>
@@ -4495,7 +4489,7 @@
         <v>20</v>
       </c>
       <c r="S22" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="T22" t="s" s="2">
         <v>20</v>
@@ -4510,13 +4504,13 @@
         <v>20</v>
       </c>
       <c r="X22" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Y22" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="Z22" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="AA22" t="s" s="2">
         <v>20</v>
@@ -4534,7 +4528,7 @@
         <v>20</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>87</v>
@@ -4549,7 +4543,7 @@
         <v>99</v>
       </c>
       <c r="AK22" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AL22" t="s" s="2">
         <v>20</v>
@@ -4563,10 +4557,10 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -4589,19 +4583,19 @@
         <v>88</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="O23" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="P23" t="s" s="2">
         <v>20</v>
@@ -4626,29 +4620,29 @@
         <v>20</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="Y23" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="Z23" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AB23" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AC23" s="2"/>
       <c r="AD23" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE23" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>78</v>
@@ -4669,7 +4663,7 @@
         <v>20</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AN23" t="s" s="2">
         <v>20</v>
@@ -4677,13 +4671,13 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C24" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D24" t="s" s="2">
         <v>20</v>
@@ -4705,19 +4699,19 @@
         <v>88</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="O24" t="s" s="2">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>20</v>
@@ -4727,7 +4721,7 @@
         <v>20</v>
       </c>
       <c r="S24" t="s" s="2">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="T24" t="s" s="2">
         <v>20</v>
@@ -4742,13 +4736,13 @@
         <v>20</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="Y24" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="Z24" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>20</v>
@@ -4766,7 +4760,7 @@
         <v>20</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>78</v>
@@ -4787,7 +4781,7 @@
         <v>20</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AN24" t="s" s="2">
         <v>20</v>
@@ -4795,10 +4789,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4821,13 +4815,13 @@
         <v>88</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -4878,7 +4872,7 @@
         <v>20</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>78</v>
@@ -4907,10 +4901,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4933,17 +4927,17 @@
         <v>88</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" t="s" s="2">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>20</v>
@@ -4992,7 +4986,7 @@
         <v>20</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>78</v>
@@ -5013,7 +5007,7 @@
         <v>20</v>
       </c>
       <c r="AM26" t="s" s="2">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="AN26" t="s" s="2">
         <v>20</v>
@@ -5021,14 +5015,14 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
@@ -5047,17 +5041,17 @@
         <v>88</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" t="s" s="2">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="P27" t="s" s="2">
         <v>20</v>
@@ -5106,7 +5100,7 @@
         <v>20</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>87</v>
@@ -5121,24 +5115,24 @@
         <v>99</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="AN27" t="s" s="2">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -5161,16 +5155,16 @@
         <v>88</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -5220,7 +5214,7 @@
         <v>20</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
@@ -5235,28 +5229,28 @@
         <v>99</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="AN28" t="s" s="2">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
@@ -5275,19 +5269,19 @@
         <v>88</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="O29" t="s" s="2">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>20</v>
@@ -5336,7 +5330,7 @@
         <v>20</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>78</v>
@@ -5351,24 +5345,24 @@
         <v>99</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="AN29" t="s" s="2">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -5391,13 +5385,13 @@
         <v>20</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -5448,7 +5442,7 @@
         <v>20</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
@@ -5466,7 +5460,7 @@
         <v>20</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AM30" t="s" s="2">
         <v>20</v>
@@ -5477,14 +5471,14 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
@@ -5503,16 +5497,16 @@
         <v>20</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="N31" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
@@ -5550,19 +5544,19 @@
         <v>20</v>
       </c>
       <c r="AB31" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AC31" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AD31" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE31" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
@@ -5574,13 +5568,13 @@
         <v>20</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AK31" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AM31" t="s" s="2">
         <v>20</v>
@@ -5591,10 +5585,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5617,16 +5611,16 @@
         <v>88</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
@@ -5676,7 +5670,7 @@
         <v>20</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>78</v>
@@ -5685,7 +5679,7 @@
         <v>87</v>
       </c>
       <c r="AI32" t="s" s="2">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="AJ32" t="s" s="2">
         <v>99</v>
@@ -5694,21 +5688,21 @@
         <v>20</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="AM32" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AN32" t="s" s="2">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5731,23 +5725,23 @@
         <v>88</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
         <v>20</v>
       </c>
       <c r="Q33" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="R33" t="s" s="2">
         <v>20</v>
@@ -5792,7 +5786,7 @@
         <v>20</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>78</v>
@@ -5801,7 +5795,7 @@
         <v>87</v>
       </c>
       <c r="AI33" t="s" s="2">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="AJ33" t="s" s="2">
         <v>99</v>
@@ -5810,25 +5804,25 @@
         <v>20</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AM33" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AN33" t="s" s="2">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
@@ -5847,13 +5841,13 @@
         <v>88</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -5904,7 +5898,7 @@
         <v>20</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>78</v>
@@ -5919,13 +5913,13 @@
         <v>99</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="AN34" t="s" s="2">
         <v>20</v>
@@ -5933,10 +5927,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5959,16 +5953,16 @@
         <v>88</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>311</v>
+        <v>197</v>
       </c>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
@@ -6018,7 +6012,7 @@
         <v>20</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>78</v>
@@ -6033,13 +6027,13 @@
         <v>99</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="AL35" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="AN35" t="s" s="2">
         <v>20</v>
@@ -6047,10 +6041,10 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -6073,16 +6067,16 @@
         <v>20</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>317</v>
+        <v>197</v>
       </c>
       <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
@@ -6132,7 +6126,7 @@
         <v>20</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>78</v>
@@ -6195,7 +6189,9 @@
       <c r="M37" t="s" s="2">
         <v>321</v>
       </c>
-      <c r="N37" s="2"/>
+      <c r="N37" t="s" s="2">
+        <v>197</v>
+      </c>
       <c r="O37" t="s" s="2">
         <v>322</v>
       </c>
@@ -6310,10 +6306,10 @@
         <v>328</v>
       </c>
       <c r="N38" t="s" s="2">
+        <v>197</v>
+      </c>
+      <c r="O38" t="s" s="2">
         <v>329</v>
-      </c>
-      <c r="O38" t="s" s="2">
-        <v>330</v>
       </c>
       <c r="P38" t="s" s="2">
         <v>20</v>
@@ -6377,24 +6373,24 @@
         <v>99</v>
       </c>
       <c r="AK38" t="s" s="2">
+        <v>330</v>
+      </c>
+      <c r="AL38" t="s" s="2">
         <v>331</v>
       </c>
-      <c r="AL38" t="s" s="2">
+      <c r="AM38" t="s" s="2">
         <v>332</v>
       </c>
-      <c r="AM38" t="s" s="2">
+      <c r="AN38" t="s" s="2">
         <v>333</v>
-      </c>
-      <c r="AN38" t="s" s="2">
-        <v>334</v>
       </c>
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6417,19 +6413,19 @@
         <v>20</v>
       </c>
       <c r="K39" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="L39" t="s" s="2">
         <v>336</v>
       </c>
-      <c r="L39" t="s" s="2">
+      <c r="M39" t="s" s="2">
         <v>337</v>
       </c>
-      <c r="M39" t="s" s="2">
+      <c r="N39" t="s" s="2">
         <v>338</v>
       </c>
-      <c r="N39" t="s" s="2">
+      <c r="O39" t="s" s="2">
         <v>339</v>
-      </c>
-      <c r="O39" t="s" s="2">
-        <v>340</v>
       </c>
       <c r="P39" t="s" s="2">
         <v>20</v>
@@ -6478,7 +6474,7 @@
         <v>20</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>78</v>
@@ -6493,7 +6489,7 @@
         <v>99</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="AL39" t="s" s="2">
         <v>20</v>
@@ -6507,10 +6503,10 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6533,19 +6529,19 @@
         <v>20</v>
       </c>
       <c r="K40" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="L40" t="s" s="2">
         <v>343</v>
       </c>
-      <c r="L40" t="s" s="2">
+      <c r="M40" t="s" s="2">
         <v>344</v>
       </c>
-      <c r="M40" t="s" s="2">
+      <c r="N40" t="s" s="2">
         <v>345</v>
       </c>
-      <c r="N40" t="s" s="2">
+      <c r="O40" t="s" s="2">
         <v>346</v>
-      </c>
-      <c r="O40" t="s" s="2">
-        <v>347</v>
       </c>
       <c r="P40" t="s" s="2">
         <v>20</v>
@@ -6594,7 +6590,7 @@
         <v>20</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>78</v>
@@ -6612,21 +6608,21 @@
         <v>20</v>
       </c>
       <c r="AL40" t="s" s="2">
+        <v>347</v>
+      </c>
+      <c r="AM40" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AN40" t="s" s="2">
         <v>348</v>
-      </c>
-      <c r="AM40" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AN40" t="s" s="2">
-        <v>349</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6649,17 +6645,17 @@
         <v>20</v>
       </c>
       <c r="K41" t="s" s="2">
+        <v>350</v>
+      </c>
+      <c r="L41" t="s" s="2">
         <v>351</v>
       </c>
-      <c r="L41" t="s" s="2">
+      <c r="M41" t="s" s="2">
         <v>352</v>
-      </c>
-      <c r="M41" t="s" s="2">
-        <v>353</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" t="s" s="2">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="P41" t="s" s="2">
         <v>20</v>
@@ -6708,7 +6704,7 @@
         <v>20</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
@@ -6720,13 +6716,13 @@
         <v>20</v>
       </c>
       <c r="AJ41" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="AK41" t="s" s="2">
         <v>355</v>
       </c>
-      <c r="AK41" t="s" s="2">
+      <c r="AL41" t="s" s="2">
         <v>356</v>
-      </c>
-      <c r="AL41" t="s" s="2">
-        <v>357</v>
       </c>
       <c r="AM41" t="s" s="2">
         <v>20</v>
@@ -6737,10 +6733,10 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6763,13 +6759,13 @@
         <v>20</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6820,7 +6816,7 @@
         <v>20</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>78</v>
@@ -6838,7 +6834,7 @@
         <v>20</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AM42" t="s" s="2">
         <v>20</v>
@@ -6849,14 +6845,14 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
@@ -6875,16 +6871,16 @@
         <v>20</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="N43" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
@@ -6934,7 +6930,7 @@
         <v>20</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>78</v>
@@ -6946,13 +6942,13 @@
         <v>20</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AK43" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AM43" t="s" s="2">
         <v>20</v>
@@ -6963,14 +6959,14 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
@@ -6989,19 +6985,19 @@
         <v>88</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L44" t="s" s="2">
+        <v>361</v>
+      </c>
+      <c r="M44" t="s" s="2">
         <v>362</v>
       </c>
-      <c r="M44" t="s" s="2">
-        <v>363</v>
-      </c>
       <c r="N44" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O44" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="P44" t="s" s="2">
         <v>20</v>
@@ -7050,7 +7046,7 @@
         <v>20</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>78</v>
@@ -7062,13 +7058,13 @@
         <v>20</v>
       </c>
       <c r="AJ44" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AK44" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL44" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AM44" t="s" s="2">
         <v>20</v>
@@ -7079,10 +7075,10 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -7105,16 +7101,16 @@
         <v>20</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L45" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="M45" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="M45" t="s" s="2">
+      <c r="N45" t="s" s="2">
         <v>367</v>
-      </c>
-      <c r="N45" t="s" s="2">
-        <v>368</v>
       </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
@@ -7140,14 +7136,14 @@
         <v>20</v>
       </c>
       <c r="X45" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="Y45" t="s" s="2">
+        <v>368</v>
+      </c>
+      <c r="Z45" t="s" s="2">
         <v>369</v>
       </c>
-      <c r="Z45" t="s" s="2">
-        <v>370</v>
-      </c>
       <c r="AA45" t="s" s="2">
         <v>20</v>
       </c>
@@ -7164,7 +7160,7 @@
         <v>20</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>78</v>
@@ -7193,10 +7189,10 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7219,19 +7215,19 @@
         <v>20</v>
       </c>
       <c r="K46" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="L46" t="s" s="2">
         <v>372</v>
       </c>
-      <c r="L46" t="s" s="2">
+      <c r="M46" t="s" s="2">
         <v>373</v>
       </c>
-      <c r="M46" t="s" s="2">
+      <c r="N46" t="s" s="2">
         <v>374</v>
       </c>
-      <c r="N46" t="s" s="2">
+      <c r="O46" t="s" s="2">
         <v>375</v>
-      </c>
-      <c r="O46" t="s" s="2">
-        <v>376</v>
       </c>
       <c r="P46" t="s" s="2">
         <v>20</v>
@@ -7280,7 +7276,7 @@
         <v>20</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>78</v>
@@ -7295,10 +7291,10 @@
         <v>99</v>
       </c>
       <c r="AK46" t="s" s="2">
+        <v>376</v>
+      </c>
+      <c r="AL46" t="s" s="2">
         <v>377</v>
-      </c>
-      <c r="AL46" t="s" s="2">
-        <v>378</v>
       </c>
       <c r="AM46" t="s" s="2">
         <v>20</v>
@@ -7309,10 +7305,10 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7335,19 +7331,19 @@
         <v>20</v>
       </c>
       <c r="K47" t="s" s="2">
+        <v>379</v>
+      </c>
+      <c r="L47" t="s" s="2">
         <v>380</v>
       </c>
-      <c r="L47" t="s" s="2">
+      <c r="M47" t="s" s="2">
         <v>381</v>
       </c>
-      <c r="M47" t="s" s="2">
+      <c r="N47" t="s" s="2">
         <v>382</v>
       </c>
-      <c r="N47" t="s" s="2">
+      <c r="O47" t="s" s="2">
         <v>383</v>
-      </c>
-      <c r="O47" t="s" s="2">
-        <v>384</v>
       </c>
       <c r="P47" t="s" s="2">
         <v>20</v>
@@ -7396,7 +7392,7 @@
         <v>20</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>78</v>
@@ -7414,21 +7410,21 @@
         <v>20</v>
       </c>
       <c r="AL47" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="AM47" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AN47" t="s" s="2">
         <v>385</v>
-      </c>
-      <c r="AM47" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AN47" t="s" s="2">
-        <v>386</v>
       </c>
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7451,19 +7447,19 @@
         <v>20</v>
       </c>
       <c r="K48" t="s" s="2">
+        <v>387</v>
+      </c>
+      <c r="L48" t="s" s="2">
         <v>388</v>
       </c>
-      <c r="L48" t="s" s="2">
+      <c r="M48" t="s" s="2">
         <v>389</v>
       </c>
-      <c r="M48" t="s" s="2">
+      <c r="N48" t="s" s="2">
+        <v>197</v>
+      </c>
+      <c r="O48" t="s" s="2">
         <v>390</v>
-      </c>
-      <c r="N48" t="s" s="2">
-        <v>391</v>
-      </c>
-      <c r="O48" t="s" s="2">
-        <v>392</v>
       </c>
       <c r="P48" t="s" s="2">
         <v>20</v>
@@ -7512,7 +7508,7 @@
         <v>20</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>78</v>
@@ -7521,16 +7517,16 @@
         <v>87</v>
       </c>
       <c r="AI48" t="s" s="2">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="AJ48" t="s" s="2">
         <v>99</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="AL48" t="s" s="2">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="AM48" t="s" s="2">
         <v>20</v>
@@ -7541,10 +7537,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7567,17 +7563,17 @@
         <v>20</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" t="s" s="2">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="P49" t="s" s="2">
         <v>20</v>
@@ -7626,7 +7622,7 @@
         <v>20</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>78</v>
@@ -7635,7 +7631,7 @@
         <v>87</v>
       </c>
       <c r="AI49" t="s" s="2">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="AJ49" t="s" s="2">
         <v>99</v>
@@ -7644,7 +7640,7 @@
         <v>20</v>
       </c>
       <c r="AL49" t="s" s="2">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="AM49" t="s" s="2">
         <v>20</v>
@@ -7655,10 +7651,10 @@
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7681,13 +7677,13 @@
         <v>20</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -7738,7 +7734,7 @@
         <v>20</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>78</v>
@@ -7756,7 +7752,7 @@
         <v>20</v>
       </c>
       <c r="AL50" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AM50" t="s" s="2">
         <v>20</v>
@@ -7767,10 +7763,10 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7793,13 +7789,13 @@
         <v>20</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
@@ -7838,17 +7834,17 @@
         <v>20</v>
       </c>
       <c r="AB51" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="AC51" s="2"/>
       <c r="AD51" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE51" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>78</v>
@@ -7860,7 +7856,7 @@
         <v>20</v>
       </c>
       <c r="AJ51" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AK51" t="s" s="2">
         <v>20</v>
@@ -7877,13 +7873,13 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C52" t="s" s="2">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="D52" t="s" s="2">
         <v>20</v>
@@ -7905,13 +7901,13 @@
         <v>20</v>
       </c>
       <c r="K52" t="s" s="2">
+        <v>404</v>
+      </c>
+      <c r="L52" t="s" s="2">
+        <v>405</v>
+      </c>
+      <c r="M52" t="s" s="2">
         <v>406</v>
-      </c>
-      <c r="L52" t="s" s="2">
-        <v>407</v>
-      </c>
-      <c r="M52" t="s" s="2">
-        <v>408</v>
       </c>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
@@ -7962,7 +7958,7 @@
         <v>20</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>78</v>
@@ -7971,10 +7967,10 @@
         <v>79</v>
       </c>
       <c r="AI52" t="s" s="2">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="AJ52" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AK52" t="s" s="2">
         <v>20</v>
@@ -7991,14 +7987,14 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E53" s="2"/>
       <c r="F53" t="s" s="2">
@@ -8017,19 +8013,19 @@
         <v>88</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L53" t="s" s="2">
+        <v>361</v>
+      </c>
+      <c r="M53" t="s" s="2">
         <v>362</v>
       </c>
-      <c r="M53" t="s" s="2">
-        <v>363</v>
-      </c>
       <c r="N53" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O53" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="P53" t="s" s="2">
         <v>20</v>
@@ -8078,7 +8074,7 @@
         <v>20</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>78</v>
@@ -8090,13 +8086,13 @@
         <v>20</v>
       </c>
       <c r="AJ53" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AK53" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AL53" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AM53" t="s" s="2">
         <v>20</v>
@@ -8107,10 +8103,10 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -8136,14 +8132,14 @@
         <v>107</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" t="s" s="2">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="P54" t="s" s="2">
         <v>20</v>
@@ -8168,13 +8164,13 @@
         <v>20</v>
       </c>
       <c r="X54" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Y54" t="s" s="2">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="Z54" t="s" s="2">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="AA54" t="s" s="2">
         <v>20</v>
@@ -8192,7 +8188,7 @@
         <v>20</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>78</v>
@@ -8210,7 +8206,7 @@
         <v>20</v>
       </c>
       <c r="AL54" t="s" s="2">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="AM54" t="s" s="2">
         <v>20</v>
@@ -8221,10 +8217,10 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8247,17 +8243,17 @@
         <v>20</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" t="s" s="2">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="P55" t="s" s="2">
         <v>20</v>
@@ -8306,7 +8302,7 @@
         <v>20</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>78</v>
@@ -8321,10 +8317,10 @@
         <v>99</v>
       </c>
       <c r="AK55" t="s" s="2">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="AL55" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AM55" t="s" s="2">
         <v>20</v>
@@ -8335,10 +8331,10 @@
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8364,16 +8360,16 @@
         <v>101</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="N56" t="s" s="2">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="O56" t="s" s="2">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="P56" t="s" s="2">
         <v>20</v>
@@ -8422,7 +8418,7 @@
         <v>20</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>78</v>
@@ -8437,10 +8433,10 @@
         <v>99</v>
       </c>
       <c r="AK56" t="s" s="2">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="AL56" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AM56" t="s" s="2">
         <v>20</v>
@@ -8451,10 +8447,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8477,19 +8473,19 @@
         <v>20</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L57" t="s" s="2">
+        <v>423</v>
+      </c>
+      <c r="M57" t="s" s="2">
+        <v>424</v>
+      </c>
+      <c r="N57" t="s" s="2">
         <v>425</v>
       </c>
-      <c r="M57" t="s" s="2">
+      <c r="O57" t="s" s="2">
         <v>426</v>
-      </c>
-      <c r="N57" t="s" s="2">
-        <v>427</v>
-      </c>
-      <c r="O57" t="s" s="2">
-        <v>428</v>
       </c>
       <c r="P57" t="s" s="2">
         <v>20</v>
@@ -8514,13 +8510,13 @@
         <v>20</v>
       </c>
       <c r="X57" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="Y57" t="s" s="2">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="Z57" t="s" s="2">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="AA57" t="s" s="2">
         <v>20</v>
@@ -8538,7 +8534,7 @@
         <v>20</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>78</v>
@@ -8553,24 +8549,24 @@
         <v>99</v>
       </c>
       <c r="AK57" t="s" s="2">
+        <v>429</v>
+      </c>
+      <c r="AL57" t="s" s="2">
+        <v>430</v>
+      </c>
+      <c r="AM57" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AN57" t="s" s="2">
         <v>431</v>
-      </c>
-      <c r="AL57" t="s" s="2">
-        <v>432</v>
-      </c>
-      <c r="AM57" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AN57" t="s" s="2">
-        <v>433</v>
       </c>
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -8593,16 +8589,16 @@
         <v>20</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L58" t="s" s="2">
+        <v>433</v>
+      </c>
+      <c r="M58" t="s" s="2">
+        <v>434</v>
+      </c>
+      <c r="N58" t="s" s="2">
         <v>435</v>
-      </c>
-      <c r="M58" t="s" s="2">
-        <v>436</v>
-      </c>
-      <c r="N58" t="s" s="2">
-        <v>437</v>
       </c>
       <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
@@ -8628,13 +8624,13 @@
         <v>20</v>
       </c>
       <c r="X58" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="Y58" t="s" s="2">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="Z58" t="s" s="2">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="AA58" t="s" s="2">
         <v>20</v>
@@ -8652,7 +8648,7 @@
         <v>20</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>78</v>
@@ -8667,7 +8663,7 @@
         <v>99</v>
       </c>
       <c r="AK58" t="s" s="2">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="AL58" t="s" s="2">
         <v>20</v>
@@ -8681,10 +8677,10 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -8707,16 +8703,16 @@
         <v>20</v>
       </c>
       <c r="K59" t="s" s="2">
+        <v>440</v>
+      </c>
+      <c r="L59" t="s" s="2">
+        <v>441</v>
+      </c>
+      <c r="M59" t="s" s="2">
         <v>442</v>
       </c>
-      <c r="L59" t="s" s="2">
+      <c r="N59" t="s" s="2">
         <v>443</v>
-      </c>
-      <c r="M59" t="s" s="2">
-        <v>444</v>
-      </c>
-      <c r="N59" t="s" s="2">
-        <v>445</v>
       </c>
       <c r="O59" s="2"/>
       <c r="P59" t="s" s="2">
@@ -8766,7 +8762,7 @@
         <v>20</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>78</v>
@@ -8781,7 +8777,7 @@
         <v>99</v>
       </c>
       <c r="AK59" t="s" s="2">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="AL59" t="s" s="2">
         <v>20</v>
@@ -8795,10 +8791,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -8821,17 +8817,17 @@
         <v>20</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="N60" s="2"/>
       <c r="O60" t="s" s="2">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="P60" t="s" s="2">
         <v>20</v>
@@ -8880,7 +8876,7 @@
         <v>20</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>78</v>
@@ -8898,7 +8894,7 @@
         <v>20</v>
       </c>
       <c r="AL60" t="s" s="2">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="AM60" t="s" s="2">
         <v>20</v>
@@ -8909,10 +8905,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -8938,16 +8934,16 @@
         <v>107</v>
       </c>
       <c r="L61" t="s" s="2">
+        <v>449</v>
+      </c>
+      <c r="M61" t="s" s="2">
+        <v>450</v>
+      </c>
+      <c r="N61" t="s" s="2">
         <v>451</v>
       </c>
-      <c r="M61" t="s" s="2">
+      <c r="O61" t="s" s="2">
         <v>452</v>
-      </c>
-      <c r="N61" t="s" s="2">
-        <v>453</v>
-      </c>
-      <c r="O61" t="s" s="2">
-        <v>454</v>
       </c>
       <c r="P61" t="s" s="2">
         <v>20</v>
@@ -8972,13 +8968,13 @@
         <v>20</v>
       </c>
       <c r="X61" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Y61" t="s" s="2">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="Z61" t="s" s="2">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="AA61" t="s" s="2">
         <v>20</v>
@@ -8996,7 +8992,7 @@
         <v>20</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>87</v>
@@ -9011,24 +9007,24 @@
         <v>99</v>
       </c>
       <c r="AK61" t="s" s="2">
+        <v>455</v>
+      </c>
+      <c r="AL61" t="s" s="2">
+        <v>456</v>
+      </c>
+      <c r="AM61" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AN61" t="s" s="2">
         <v>457</v>
-      </c>
-      <c r="AL61" t="s" s="2">
-        <v>458</v>
-      </c>
-      <c r="AM61" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AN61" t="s" s="2">
-        <v>459</v>
       </c>
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -9051,16 +9047,16 @@
         <v>20</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L62" t="s" s="2">
+        <v>459</v>
+      </c>
+      <c r="M62" t="s" s="2">
+        <v>460</v>
+      </c>
+      <c r="N62" t="s" s="2">
         <v>461</v>
-      </c>
-      <c r="M62" t="s" s="2">
-        <v>462</v>
-      </c>
-      <c r="N62" t="s" s="2">
-        <v>463</v>
       </c>
       <c r="O62" s="2"/>
       <c r="P62" t="s" s="2">
@@ -9110,7 +9106,7 @@
         <v>20</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>78</v>
@@ -9125,7 +9121,7 @@
         <v>99</v>
       </c>
       <c r="AK62" t="s" s="2">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="AL62" t="s" s="2">
         <v>20</v>
@@ -9139,10 +9135,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -9165,26 +9161,26 @@
         <v>20</v>
       </c>
       <c r="K63" t="s" s="2">
+        <v>464</v>
+      </c>
+      <c r="L63" t="s" s="2">
+        <v>465</v>
+      </c>
+      <c r="M63" t="s" s="2">
         <v>466</v>
       </c>
-      <c r="L63" t="s" s="2">
+      <c r="N63" t="s" s="2">
         <v>467</v>
       </c>
-      <c r="M63" t="s" s="2">
+      <c r="O63" t="s" s="2">
         <v>468</v>
       </c>
-      <c r="N63" t="s" s="2">
+      <c r="P63" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="Q63" t="s" s="2">
         <v>469</v>
       </c>
-      <c r="O63" t="s" s="2">
-        <v>470</v>
-      </c>
-      <c r="P63" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="Q63" t="s" s="2">
-        <v>471</v>
-      </c>
       <c r="R63" t="s" s="2">
         <v>20</v>
       </c>
@@ -9228,7 +9224,7 @@
         <v>20</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>78</v>
@@ -9243,10 +9239,10 @@
         <v>99</v>
       </c>
       <c r="AK63" t="s" s="2">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="AL63" t="s" s="2">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="AM63" t="s" s="2">
         <v>20</v>
@@ -9257,10 +9253,10 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9283,17 +9279,17 @@
         <v>20</v>
       </c>
       <c r="K64" t="s" s="2">
+        <v>473</v>
+      </c>
+      <c r="L64" t="s" s="2">
+        <v>474</v>
+      </c>
+      <c r="M64" t="s" s="2">
         <v>475</v>
-      </c>
-      <c r="L64" t="s" s="2">
-        <v>476</v>
-      </c>
-      <c r="M64" t="s" s="2">
-        <v>477</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" t="s" s="2">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="P64" t="s" s="2">
         <v>20</v>
@@ -9330,17 +9326,17 @@
         <v>20</v>
       </c>
       <c r="AB64" t="s" s="2">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="AC64" s="2"/>
       <c r="AD64" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE64" t="s" s="2">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>78</v>
@@ -9355,27 +9351,27 @@
         <v>99</v>
       </c>
       <c r="AK64" t="s" s="2">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="AL64" t="s" s="2">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="AM64" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AN64" t="s" s="2">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="C65" t="s" s="2">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="D65" t="s" s="2">
         <v>20</v>
@@ -9397,17 +9393,17 @@
         <v>20</v>
       </c>
       <c r="K65" t="s" s="2">
+        <v>473</v>
+      </c>
+      <c r="L65" t="s" s="2">
+        <v>474</v>
+      </c>
+      <c r="M65" t="s" s="2">
         <v>475</v>
-      </c>
-      <c r="L65" t="s" s="2">
-        <v>476</v>
-      </c>
-      <c r="M65" t="s" s="2">
-        <v>477</v>
       </c>
       <c r="N65" s="2"/>
       <c r="O65" t="s" s="2">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="P65" t="s" s="2">
         <v>20</v>
@@ -9456,7 +9452,7 @@
         <v>20</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>78</v>
@@ -9471,24 +9467,24 @@
         <v>99</v>
       </c>
       <c r="AK65" t="s" s="2">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="AL65" t="s" s="2">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="AM65" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AN65" t="s" s="2">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -9511,19 +9507,19 @@
         <v>20</v>
       </c>
       <c r="K66" t="s" s="2">
+        <v>483</v>
+      </c>
+      <c r="L66" t="s" s="2">
+        <v>484</v>
+      </c>
+      <c r="M66" t="s" s="2">
         <v>485</v>
       </c>
-      <c r="L66" t="s" s="2">
+      <c r="N66" t="s" s="2">
+        <v>197</v>
+      </c>
+      <c r="O66" t="s" s="2">
         <v>486</v>
-      </c>
-      <c r="M66" t="s" s="2">
-        <v>487</v>
-      </c>
-      <c r="N66" t="s" s="2">
-        <v>488</v>
-      </c>
-      <c r="O66" t="s" s="2">
-        <v>489</v>
       </c>
       <c r="P66" t="s" s="2">
         <v>20</v>
@@ -9572,7 +9568,7 @@
         <v>20</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="AG66" t="s" s="2">
         <v>78</v>
@@ -9590,21 +9586,21 @@
         <v>20</v>
       </c>
       <c r="AL66" t="s" s="2">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="AM66" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AN66" t="s" s="2">
-        <v>491</v>
+        <v>488</v>
       </c>
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -9627,19 +9623,19 @@
         <v>20</v>
       </c>
       <c r="K67" t="s" s="2">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="L67" t="s" s="2">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="M67" t="s" s="2">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="N67" t="s" s="2">
-        <v>496</v>
+        <v>197</v>
       </c>
       <c r="O67" t="s" s="2">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="P67" t="s" s="2">
         <v>20</v>
@@ -9688,7 +9684,7 @@
         <v>20</v>
       </c>
       <c r="AF67" t="s" s="2">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="AG67" t="s" s="2">
         <v>78</v>
@@ -9703,24 +9699,24 @@
         <v>99</v>
       </c>
       <c r="AK67" t="s" s="2">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="AL67" t="s" s="2">
-        <v>498</v>
+        <v>494</v>
       </c>
       <c r="AM67" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AN67" t="s" s="2">
-        <v>499</v>
+        <v>495</v>
       </c>
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -9743,13 +9739,13 @@
         <v>20</v>
       </c>
       <c r="K68" t="s" s="2">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="L68" t="s" s="2">
-        <v>502</v>
+        <v>498</v>
       </c>
       <c r="M68" t="s" s="2">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
@@ -9776,29 +9772,29 @@
         <v>20</v>
       </c>
       <c r="X68" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="Y68" t="s" s="2">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="Z68" t="s" s="2">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="AA68" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AB68" t="s" s="2">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="AC68" s="2"/>
       <c r="AD68" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AE68" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>78</v>
@@ -9816,24 +9812,24 @@
         <v>20</v>
       </c>
       <c r="AL68" t="s" s="2">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="AM68" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AN68" t="s" s="2">
-        <v>507</v>
+        <v>503</v>
       </c>
     </row>
     <row r="69" hidden="true">
       <c r="A69" t="s" s="2">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="C69" t="s" s="2">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="D69" t="s" s="2">
         <v>20</v>
@@ -9855,15 +9851,17 @@
         <v>20</v>
       </c>
       <c r="K69" t="s" s="2">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="L69" t="s" s="2">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="M69" t="s" s="2">
-        <v>503</v>
-      </c>
-      <c r="N69" s="2"/>
+        <v>508</v>
+      </c>
+      <c r="N69" t="s" s="2">
+        <v>197</v>
+      </c>
       <c r="O69" s="2"/>
       <c r="P69" t="s" s="2">
         <v>20</v>
@@ -9912,7 +9910,7 @@
         <v>20</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>78</v>
@@ -9930,25 +9928,25 @@
         <v>20</v>
       </c>
       <c r="AL69" t="s" s="2">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="AM69" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AN69" t="s" s="2">
-        <v>507</v>
+        <v>503</v>
       </c>
     </row>
     <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="E70" s="2"/>
       <c r="F70" t="s" s="2">
@@ -9967,17 +9965,17 @@
         <v>20</v>
       </c>
       <c r="K70" t="s" s="2">
+        <v>511</v>
+      </c>
+      <c r="L70" t="s" s="2">
+        <v>512</v>
+      </c>
+      <c r="M70" t="s" s="2">
         <v>513</v>
-      </c>
-      <c r="L70" t="s" s="2">
-        <v>514</v>
-      </c>
-      <c r="M70" t="s" s="2">
-        <v>515</v>
       </c>
       <c r="N70" s="2"/>
       <c r="O70" t="s" s="2">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="P70" t="s" s="2">
         <v>20</v>
@@ -10026,7 +10024,7 @@
         <v>20</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>78</v>
@@ -10044,21 +10042,21 @@
         <v>20</v>
       </c>
       <c r="AL70" t="s" s="2">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="AM70" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AN70" t="s" s="2">
-        <v>518</v>
+        <v>516</v>
       </c>
     </row>
     <row r="71" hidden="true">
       <c r="A71" t="s" s="2">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -10081,13 +10079,13 @@
         <v>20</v>
       </c>
       <c r="K71" t="s" s="2">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
@@ -10138,7 +10136,7 @@
         <v>20</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>78</v>
@@ -10156,21 +10154,21 @@
         <v>20</v>
       </c>
       <c r="AL71" t="s" s="2">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="AM71" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AN71" t="s" s="2">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -10193,13 +10191,13 @@
         <v>20</v>
       </c>
       <c r="K72" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
@@ -10250,7 +10248,7 @@
         <v>20</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>78</v>
@@ -10268,21 +10266,21 @@
         <v>20</v>
       </c>
       <c r="AL72" t="s" s="2">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="AM72" t="s" s="2">
         <v>20</v>
       </c>
       <c r="AN72" t="s" s="2">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -10305,17 +10303,17 @@
         <v>20</v>
       </c>
       <c r="K73" t="s" s="2">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="L73" t="s" s="2">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="M73" t="s" s="2">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="N73" s="2"/>
       <c r="O73" t="s" s="2">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="P73" t="s" s="2">
         <v>20</v>
@@ -10364,7 +10362,7 @@
         <v>20</v>
       </c>
       <c r="AF73" t="s" s="2">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="AG73" t="s" s="2">
         <v>78</v>
@@ -10379,16 +10377,16 @@
         <v>99</v>
       </c>
       <c r="AK73" t="s" s="2">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="AL73" t="s" s="2">
+        <v>384</v>
+      </c>
+      <c r="AM73" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="AN73" t="s" s="2">
         <v>385</v>
-      </c>
-      <c r="AM73" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="AN73" t="s" s="2">
-        <v>386</v>
       </c>
     </row>
   </sheetData>

</xml_diff>